<commit_message>
Add targets, status colors, intro report and Streamlit app (pre-v2 draft)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/examples/sample_contacts.xlsx
+++ b/examples/sample_contacts.xlsx
@@ -1,14 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Contacts" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="How to use" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Contacts" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Targets" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="How to use" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Contacts'!$A$1:$I$23</definedName>
@@ -61,11 +62,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
@@ -1211,7 +1213,93 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B11"/>
+  <dimension ref="A1:B6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="50" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>Company</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Northwind Consulting</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Strategy practice</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Summit Airlines</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Pinecrest Labs</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Reachable only through Liam</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Granite Peak Partners</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>No one yet</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Harborview Media</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>No one yet</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1219,124 +1307,136 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="inlineStr">
+      <c r="A1" s="3" t="inlineStr">
         <is>
           <t>Name</t>
         </is>
       </c>
-      <c r="B1" s="3" t="inlineStr">
+      <c r="B1" s="4" t="inlineStr">
         <is>
           <t>Required. Full name, spelled the same way everywhere.</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" s="3" t="inlineStr">
         <is>
           <t>Company</t>
         </is>
       </c>
-      <c r="B2" s="3" t="inlineStr">
+      <c r="B2" s="4" t="inlineStr">
         <is>
           <t>Current company. 3+ direct connections at one company become a group.</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+      <c r="A3" s="3" t="inlineStr">
         <is>
           <t>School</t>
         </is>
       </c>
-      <c r="B3" s="3" t="inlineStr">
+      <c r="B3" s="4" t="inlineStr">
         <is>
           <t>School they attended. 3+ at one school become a group. 'BYU' and 'Brigham Young University' count as the same.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="inlineStr">
+      <c r="A4" s="3" t="inlineStr">
         <is>
           <t>Role</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B4" s="4" t="inlineStr">
         <is>
           <t>Job title (optional).</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="inlineStr">
+      <c r="A5" s="3" t="inlineStr">
         <is>
           <t>Connected Through</t>
         </is>
       </c>
-      <c r="B5" s="3" t="inlineStr">
+      <c r="B5" s="4" t="inlineStr">
         <is>
           <t>Leave BLANK if you know them directly. If someone introduced you (or you know OF them through someone), put that person's name here and they appear as a 2nd-degree connection.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="inlineStr">
+      <c r="A6" s="3" t="inlineStr">
         <is>
           <t>LinkedIn URL</t>
         </is>
       </c>
-      <c r="B6" s="3" t="inlineStr">
+      <c r="B6" s="4" t="inlineStr">
         <is>
           <t>Paste their profile link. Double-click them on the map to open it.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="inlineStr">
+      <c r="A7" s="3" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="B7" s="3" t="inlineStr">
+      <c r="B7" s="4" t="inlineStr">
         <is>
           <t>Met / To Reach Out / Contacted / Follow Up / Referral.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="inlineStr">
+      <c r="A8" s="3" t="inlineStr">
         <is>
           <t>Tags</t>
         </is>
       </c>
-      <c r="B8" s="3" t="inlineStr">
+      <c r="B8" s="4" t="inlineStr">
         <is>
           <t>Optional, comma-separated (e.g. 'MCA, Delta recruiting'). Group by tags with: --group-by company,school,tags</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="inlineStr">
+      <c r="A9" s="3" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
-      <c r="B9" s="3" t="inlineStr">
+      <c r="B9" s="4" t="inlineStr">
         <is>
           <t>Anything you want to remember.</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="2" t="inlineStr"/>
-      <c r="B10" s="3" t="inlineStr"/>
+      <c r="A10" s="3" t="inlineStr"/>
+      <c r="B10" s="4" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="A11" s="2" t="inlineStr">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>Targets tab</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>List companies you want to work at (one per row). Targets are outlined in red on the map; ones with no connections show as hollow red bubbles, and build_map.py writes a 'who can intro me?' report for each.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
         <is>
           <t>LinkedIn export</t>
         </is>
       </c>
-      <c r="B11" s="3" t="inlineStr">
+      <c r="B12" s="4" t="inlineStr">
         <is>
           <t>LinkedIn &gt; Settings &gt; Data privacy &gt; Get a copy of your data &gt; Connections. Pass the Connections.csv with --linkedin. Rows here with the same name override the export (so you can add schools).</t>
         </is>

</xml_diff>